<commit_message>
fix data mapping columns, normalize station names, remove previous week carryover, improve heatmap scroll z-index and row hover
</commit_message>
<xml_diff>
--- a/data/weeks/ANM_PS_04_06_2026-10_06_2026.xlsx
+++ b/data/weeks/ANM_PS_04_06_2026-10_06_2026.xlsx
@@ -638,7 +638,7 @@
         <v>100</v>
       </c>
       <c r="M3" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
         <v>100</v>
@@ -647,10 +647,10 @@
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>100</v>
+        <v>96.551724137931</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -708,19 +708,19 @@
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N4" t="n">
         <v>0</v>
       </c>
       <c r="O4" t="n">
-        <v>0</v>
+        <v>16.2280701754386</v>
       </c>
       <c r="P4" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>100</v>
+        <v>98.7179487179487</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -778,7 +778,7 @@
         <v>100</v>
       </c>
       <c r="M5" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
         <v>0</v>
@@ -787,7 +787,7 @@
         <v>0</v>
       </c>
       <c r="P5" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="n">
         <v>100</v>
@@ -848,19 +848,19 @@
         <v>0</v>
       </c>
       <c r="M6" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N6" t="n">
         <v>5</v>
       </c>
       <c r="O6" t="n">
-        <v>0</v>
+        <v>23.6714975845411</v>
       </c>
       <c r="P6" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>100</v>
+        <v>98.8372093023256</v>
       </c>
       <c r="R6" t="n">
         <v>0</v>
@@ -918,16 +918,16 @@
         <v>100</v>
       </c>
       <c r="M7" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N7" t="n">
         <v>15</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>21.7391304347826</v>
       </c>
       <c r="P7" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q7" t="n">
         <v>100</v>
@@ -988,16 +988,16 @@
         <v>100</v>
       </c>
       <c r="M8" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
         <v>10</v>
       </c>
       <c r="O8" t="n">
-        <v>0</v>
+        <v>4.27350427350428</v>
       </c>
       <c r="P8" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q8" t="n">
         <v>100</v>
@@ -1058,19 +1058,19 @@
         <v>100</v>
       </c>
       <c r="M9" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N9" t="n">
         <v>0</v>
       </c>
       <c r="O9" t="n">
-        <v>0</v>
+        <v>17.2268907563025</v>
       </c>
       <c r="P9" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q9" t="n">
-        <v>100</v>
+        <v>96.2962962962963</v>
       </c>
       <c r="R9" t="n">
         <v>0</v>
@@ -1128,19 +1128,19 @@
         <v>100</v>
       </c>
       <c r="M10" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
         <v>0</v>
       </c>
       <c r="O10" t="n">
-        <v>0</v>
+        <v>1.26582278481012</v>
       </c>
       <c r="P10" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>100</v>
+        <v>94.11764705882349</v>
       </c>
       <c r="R10" t="n">
         <v>0</v>
@@ -1198,19 +1198,19 @@
         <v>100</v>
       </c>
       <c r="M11" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N11" t="n">
         <v>0</v>
       </c>
       <c r="O11" t="n">
-        <v>0</v>
+        <v>1.22950819672131</v>
       </c>
       <c r="P11" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>100</v>
+        <v>97.61904761904761</v>
       </c>
       <c r="R11" t="n">
         <v>0</v>
@@ -1268,19 +1268,19 @@
         <v>100</v>
       </c>
       <c r="M12" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N12" t="n">
         <v>10</v>
       </c>
       <c r="O12" t="n">
-        <v>0</v>
+        <v>18.3783783783784</v>
       </c>
       <c r="P12" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>100</v>
+        <v>85.4166666666667</v>
       </c>
       <c r="R12" t="n">
         <v>0</v>
@@ -1338,19 +1338,19 @@
         <v>100</v>
       </c>
       <c r="M13" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N13" t="n">
         <v>10</v>
       </c>
       <c r="O13" t="n">
-        <v>0</v>
+        <v>1.47058823529412</v>
       </c>
       <c r="P13" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="R13" t="n">
         <v>0</v>
@@ -1408,7 +1408,7 @@
         <v>100</v>
       </c>
       <c r="M14" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
         <v>5</v>
@@ -1417,10 +1417,10 @@
         <v>0</v>
       </c>
       <c r="P14" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>100</v>
+        <v>97.5</v>
       </c>
       <c r="R14" t="n">
         <v>0</v>
@@ -1457,10 +1457,10 @@
         <v>100</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>18.9410331280167</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>41.1764705882353</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -1472,37 +1472,37 @@
         <v>100</v>
       </c>
       <c r="K15" t="n">
-        <v>100</v>
+        <v>85.71428571428569</v>
       </c>
       <c r="L15" t="n">
         <v>100</v>
       </c>
       <c r="M15" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
         <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>0</v>
+        <v>1.36986301369863</v>
       </c>
       <c r="P15" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q15" t="n">
         <v>100</v>
       </c>
       <c r="R15" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>100</v>
+        <v>66.6666666666667</v>
       </c>
       <c r="T15" t="n">
-        <v>100</v>
+        <v>3.90243902439024</v>
       </c>
       <c r="U15" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="V15" t="n">
         <v>0</v>
@@ -1548,19 +1548,19 @@
         <v>0</v>
       </c>
       <c r="M16" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N16" t="n">
         <v>25</v>
       </c>
       <c r="O16" t="n">
-        <v>0</v>
+        <v>24.8717948717949</v>
       </c>
       <c r="P16" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>100</v>
+        <v>97.27272727272729</v>
       </c>
       <c r="R16" t="n">
         <v>0</v>
@@ -1618,7 +1618,7 @@
         <v>100</v>
       </c>
       <c r="M17" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N17" t="n">
         <v>10</v>
@@ -1627,7 +1627,7 @@
         <v>0</v>
       </c>
       <c r="P17" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q17" t="n">
         <v>100</v>
@@ -1688,19 +1688,19 @@
         <v>100</v>
       </c>
       <c r="M18" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N18" t="n">
         <v>0</v>
       </c>
       <c r="O18" t="n">
-        <v>0</v>
+        <v>25.9615384615384</v>
       </c>
       <c r="P18" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>100</v>
+        <v>95.4545454545455</v>
       </c>
       <c r="R18" t="n">
         <v>0</v>
@@ -1758,16 +1758,16 @@
         <v>100</v>
       </c>
       <c r="M19" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
         <v>5</v>
       </c>
       <c r="O19" t="n">
-        <v>94.2622950819672</v>
+        <v>81.9366154694799</v>
       </c>
       <c r="P19" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q19" t="n">
         <v>100</v>
@@ -1828,19 +1828,19 @@
         <v>100</v>
       </c>
       <c r="M20" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N20" t="n">
         <v>5</v>
       </c>
       <c r="O20" t="n">
-        <v>90.81081081081081</v>
+        <v>81.3926665519022</v>
       </c>
       <c r="P20" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>100</v>
+        <v>97.0588235294118</v>
       </c>
       <c r="R20" t="n">
         <v>0</v>
@@ -1898,19 +1898,19 @@
         <v>100</v>
       </c>
       <c r="M21" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N21" t="n">
         <v>5</v>
       </c>
       <c r="O21" t="n">
-        <v>0</v>
+        <v>27.8947368421052</v>
       </c>
       <c r="P21" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>100</v>
+        <v>98.14814814814819</v>
       </c>
       <c r="R21" t="n">
         <v>0</v>
@@ -1968,16 +1968,16 @@
         <v>100</v>
       </c>
       <c r="M22" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N22" t="n">
         <v>5</v>
       </c>
       <c r="O22" t="n">
-        <v>0</v>
+        <v>1.10410094637224</v>
       </c>
       <c r="P22" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q22" t="n">
         <v>100</v>
@@ -2038,19 +2038,19 @@
         <v>100</v>
       </c>
       <c r="M23" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N23" t="n">
         <v>0</v>
       </c>
       <c r="O23" t="n">
-        <v>0</v>
+        <v>31.3291139240506</v>
       </c>
       <c r="P23" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>100</v>
+        <v>97.0588235294118</v>
       </c>
       <c r="R23" t="n">
         <v>0</v>
@@ -2108,19 +2108,19 @@
         <v>100</v>
       </c>
       <c r="M24" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N24" t="n">
         <v>0</v>
       </c>
       <c r="O24" t="n">
-        <v>98.10606060606059</v>
+        <v>93.0795789755966</v>
       </c>
       <c r="P24" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>100</v>
+        <v>94.11764705882349</v>
       </c>
       <c r="R24" t="n">
         <v>0</v>
@@ -2178,7 +2178,7 @@
         <v>100</v>
       </c>
       <c r="M25" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N25" t="n">
         <v>5</v>
@@ -2187,7 +2187,7 @@
         <v>0</v>
       </c>
       <c r="P25" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q25" t="n">
         <v>100</v>
@@ -2248,16 +2248,16 @@
         <v>100</v>
       </c>
       <c r="M26" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N26" t="n">
         <v>0</v>
       </c>
       <c r="O26" t="n">
-        <v>0</v>
+        <v>3.53535353535353</v>
       </c>
       <c r="P26" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q26" t="n">
         <v>100</v>
@@ -2318,16 +2318,16 @@
         <v>100</v>
       </c>
       <c r="M27" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N27" t="n">
         <v>15</v>
       </c>
       <c r="O27" t="n">
-        <v>93.5251798561151</v>
+        <v>91.1174286377349</v>
       </c>
       <c r="P27" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q27" t="n">
         <v>100</v>
@@ -2388,16 +2388,16 @@
         <v>100</v>
       </c>
       <c r="M28" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N28" t="n">
         <v>5</v>
       </c>
       <c r="O28" t="n">
-        <v>0</v>
+        <v>31.0483870967742</v>
       </c>
       <c r="P28" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q28" t="n">
         <v>100</v>
@@ -2458,16 +2458,16 @@
         <v>100</v>
       </c>
       <c r="M29" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N29" t="n">
         <v>10</v>
       </c>
       <c r="O29" t="n">
-        <v>93.1726907630522</v>
+        <v>89.44348823866891</v>
       </c>
       <c r="P29" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q29" t="n">
         <v>100</v>
@@ -2528,19 +2528,19 @@
         <v>100</v>
       </c>
       <c r="M30" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="N30" t="n">
         <v>20</v>
       </c>
       <c r="O30" t="n">
-        <v>97.5247524752475</v>
+        <v>94.68074358456251</v>
       </c>
       <c r="P30" t="n">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="Q30" t="n">
-        <v>100</v>
+        <v>93.1818181818182</v>
       </c>
       <c r="R30" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
feat: redistribute parameter weights to sum to 100% and fix admin JSON export pipeline
</commit_message>
<xml_diff>
--- a/data/weeks/ANM_PS_04_06_2026-10_06_2026.xlsx
+++ b/data/weeks/ANM_PS_04_06_2026-10_06_2026.xlsx
@@ -535,67 +535,67 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="C2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="D2" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="F2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="G2" t="n">
-        <v>0.025</v>
+        <v>0.04</v>
       </c>
       <c r="H2" t="n">
-        <v>0.025</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="J2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="K2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="L2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="M2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="N2" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="P2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="R2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="S2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="T2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="U2" t="n">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="V2" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>